<commit_message>
test: add simulator acceptance reports
</commit_message>
<xml_diff>
--- a/tests/docs/3rd-testtable.xlsx
+++ b/tests/docs/3rd-testtable.xlsx
@@ -1553,6 +1553,26 @@
           <t>量子金融算法建模工具构件测试（Func-80）</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>.venv/bin/python tests/scripts/140-quantum_finance_algorithm_modeling.py</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>tests/docs/140-quantum_finance_algorithm_modeling/results.md</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>tests/docs/140-quantum_finance_algorithm_modeling/technical_report.md</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>tests/docs/140-quantum_finance_algorithm_modeling/test_report.md</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="20" customHeight="1" s="17" thickBot="1">
       <c r="A24" s="21" t="n"/>
@@ -1576,6 +1596,26 @@
           <t>求解精度分析工具构件测试（Func-81）</t>
         </is>
       </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>.venv/bin/python tests/scripts/141-solution_precision_analysis.py</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>tests/docs/141-solution_precision_analysis/results.md</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>tests/docs/141-solution_precision_analysis/technical_report.md</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>tests/docs/141-solution_precision_analysis/test_report.md</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="20" customHeight="1" s="17" thickBot="1">
       <c r="A25" s="21" t="n"/>
@@ -1597,6 +1637,26 @@
       <c r="G25" s="3" t="inlineStr">
         <is>
           <t>计算复杂度对比分析工具构件测试（Func-82）</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>.venv/bin/python tests/scripts/142-complexity_comparison.py</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>tests/docs/142-complexity_comparison/results.md</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>tests/docs/142-complexity_comparison/technical_report.md</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>tests/docs/142-complexity_comparison/test_report.md</t>
         </is>
       </c>
     </row>
@@ -1618,6 +1678,26 @@
           <t>算法复杂度优化工具构件测试（Func-83）</t>
         </is>
       </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>.venv/bin/python tests/scripts/143-circuit_depth_optimization.py</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>tests/docs/143-circuit_depth_optimization/results.md</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>tests/docs/143-circuit_depth_optimization/technical_report.md</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>tests/docs/143-circuit_depth_optimization/test_report.md</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="20" customHeight="1" s="17" thickBot="1">
       <c r="A27" s="21" t="n"/>
@@ -1637,6 +1717,26 @@
           <t>含噪量子金融计算模拟工具构件测试（Func-84）</t>
         </is>
       </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>.venv/bin/python tests/scripts/144-noisy_quantum_finance_simulation.py</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>tests/docs/144-noisy_quantum_finance_simulation/results.md</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>tests/docs/144-noisy_quantum_finance_simulation/technical_report.md</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>tests/docs/144-noisy_quantum_finance_simulation/test_report.md</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="35" customHeight="1" s="17" thickBot="1">
       <c r="A28" s="21" t="n"/>
@@ -1654,6 +1754,26 @@
       <c r="G28" s="3" t="inlineStr">
         <is>
           <t>20比特及以上量子金融算法设计与仿真支撑能力测试（Func-85）</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>.venv/bin/python tests/scripts/145-20qubit_quantum_finance_simulation.py</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>tests/docs/145-20qubit_quantum_finance_simulation/results.md</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>tests/docs/145-20qubit_quantum_finance_simulation/technical_report.md</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>tests/docs/145-20qubit_quantum_finance_simulation/test_report.md</t>
         </is>
       </c>
     </row>

</xml_diff>